<commit_message>
Update scraped data - 2025-09-20 20:16:06 UTC
</commit_message>
<xml_diff>
--- a/2025-09-20/expected_arrival.xlsx
+++ b/2025-09-20/expected_arrival.xlsx
@@ -416,13 +416,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Updated on Saturday, 20 September 2025;</t>
+          <t>Updated on Sunday, 21 September 2025;</t>
         </is>
       </c>
     </row>
@@ -468,17 +468,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Hui Fa</t>
+          <t>Cosco New York</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Merchant Shipping (Pvt) Ltd</t>
+          <t>Cosco Shiping Line Pak Pvt Ltd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9/18/2025 12:40:00 PM</t>
+          <t>9/19/2025 9:25:00 AM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -493,24 +493,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>One Recommendation</t>
+          <t>Xin Xin Hai 2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ocean Network Express Pakistan (Pvt) Ltd</t>
+          <t>International Shipping &amp; Ports Services (Pvt) Ltd.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9/18/2025 10:05:00 PM</t>
+          <t>9/19/2025 11:00:00 AM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -525,24 +525,24 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cosco New York</t>
+          <t>Msc Veracruz V</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cosco Shiping Line Pak Pvt Ltd</t>
+          <t>Msc Agency Pakistan (Pvt) Ltd.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9/19/2025 9:25:00 AM</t>
+          <t>9/19/2025 11:05:00 AM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -557,24 +557,24 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Xin Xin Hai 2</t>
+          <t>Hong Yong Chang Sheng</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>International Shipping &amp; Ports Services (Pvt) Ltd.</t>
+          <t>Feeder Logistics</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9/19/2025 11:00:00 AM</t>
+          <t>9/19/2025 11:30:00 AM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -589,24 +589,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Msc Veracruz V</t>
+          <t>Jin Shun He</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Msc Agency Pakistan (Pvt) Ltd.</t>
+          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9/19/2025 11:05:00 AM</t>
+          <t>9/19/2025 3:00:00 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -621,24 +621,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hong Yong Chang Sheng</t>
+          <t>Kmtc Manila</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Feeder Logistics</t>
+          <t>United Marine Agencies Pvt Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>9/19/2025 11:30:00 AM</t>
+          <t>9/19/2025 10:20:00 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -653,24 +653,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jin Shun He</t>
+          <t>Msc Paloma</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
+          <t>Msc Agency Pakistan (Pvt) Ltd.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9/19/2025 3:00:00 PM</t>
+          <t>9/20/2025 11:05:00 AM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -685,24 +685,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kmtc Manila</t>
+          <t>Beijing Bridge</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>United Marine Agencies Pvt Ltd</t>
+          <t>SEA WORLD (SMC-PVT)LTD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>9/19/2025 10:20:00 PM</t>
+          <t>9/20/2025 11:15:00 AM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>9/20/2025 9:01:00 AM</t>
+          <t>9/20/2025 12:30:00 PM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -749,24 +749,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Msc Paloma</t>
+          <t>Kota Manzanillo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Msc Agency Pakistan (Pvt) Ltd.</t>
+          <t>Pacific Delta Shipping (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>9/20/2025 9:30:00 AM</t>
+          <t>9/20/2025 1:00:00 PM</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -781,24 +781,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Beijing Bridge</t>
+          <t>Apl Qingdao</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SEA WORLD (SMC-PVT)LTD</t>
+          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>9/20/2025 10:00:00 AM</t>
+          <t>9/20/2025 10:00:00 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -813,24 +813,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Kota Manzanillo</t>
+          <t>Oocl Nagoya</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pacific Delta Shipping (Pvt) Ltd</t>
+          <t>OOCL PAKISTAN (PVT) LIMITED.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>9/20/2025 1:00:00 PM</t>
+          <t>9/20/2025 10:00:00 PM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -845,24 +845,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Apl Qingdao</t>
+          <t>Ital Universo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
+          <t>GREEN PAK SHIPPING PVT LTD</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>9/20/2025 3:00:00 PM</t>
+          <t>9/21/2025 12:00:00 AM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -877,24 +877,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Oocl Nagoya</t>
+          <t>Seaspan Santos</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OOCL PAKISTAN (PVT) LIMITED.</t>
+          <t>Gac Pakistan (Pvt) Limited.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>9/20/2025 10:00:00 PM</t>
+          <t>9/21/2025 6:30:00 AM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -909,24 +909,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ital Universo</t>
+          <t>X-Press Pyxis</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GREEN PAK SHIPPING PVT LTD</t>
+          <t>X-Press Feeders Shipping Agency Pakistan (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>9/21/2025 12:00:00 AM</t>
+          <t>9/21/2025 5:00:00 PM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -941,24 +941,24 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Seaspan Santos</t>
+          <t>X-Press Kohima</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gac Pakistan (Pvt) Limited.</t>
+          <t>X-Press Feeders Shipping Agency Pakistan (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>9/21/2025 6:30:00 AM</t>
+          <t>9/21/2025 6:30:00 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -973,24 +973,24 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>X-Press Pyxis</t>
+          <t>Gfs Prime</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>X-Press Feeders Shipping Agency Pakistan (Pvt) Ltd</t>
+          <t>Eastwind Shipping Company (pvt) Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>9/21/2025 5:00:00 PM</t>
+          <t>9/21/2025 10:00:00 PM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1005,24 +1005,24 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cma Cgm Zanzibar</t>
+          <t>Kmtc Colombo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
+          <t>United Marine Agencies Pvt Ltd</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>9/21/2025 8:00:00 PM</t>
+          <t>9/22/2025 1:00:00 AM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1037,24 +1037,24 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>X-Press Kohima</t>
+          <t>Cma Cgm Zanzibar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>X-Press Feeders Shipping Agency Pakistan (Pvt) Ltd</t>
+          <t>Cma Cgm Pakistan (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>9/21/2025 9:00:00 PM</t>
+          <t>9/22/2025 11:00:00 AM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1069,24 +1069,24 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gfs Prime</t>
+          <t>Wan Hai 316</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Eastwind Shipping Company (pvt) Ltd</t>
+          <t>Riazeda (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>9/21/2025 10:00:00 PM</t>
+          <t>9/22/2025 12:00:00 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1101,24 +1101,24 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kmtc Colombo</t>
+          <t>Kai Da Hong Zhou</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>United Marine Agencies Pvt Ltd</t>
+          <t>Yaaseen Shipping Lines (Pvt) Ltd.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>9/22/2025 1:00:00 AM</t>
+          <t>9/23/2025 6:00:00 AM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1133,24 +1133,24 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wan Hai 316</t>
+          <t>Seaspan Bellwether</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Riazeda (Pvt) Ltd</t>
+          <t>United Marine Agencies Pvt Ltd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>9/22/2025 12:00:00 PM</t>
+          <t>9/23/2025 11:00:00 AM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1165,242 +1165,299 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Crude Oil</t>
+          <t>2025-09-20 20:15:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gsl Grania</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gac Pakistan (Pvt) Limited.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>9/23/2025 12:30:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Shipping Agent</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Arrival Strip</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Import(Tons)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Export(Tons)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
+          <t>Crude Oil</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>M.T.Shalamar</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pakistan National Ship.Corpt.</t>
+          <t>Shipping Agent</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>9/21/2025 11:30:00 AM</t>
+          <t>Arrival Strip</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Import(73000.0)</t>
+          <t>Import(Tons)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Export(Tons)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>M.T.Shalamar</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Pakistan National Ship.Corpt.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>9/21/2025 11:30:00 AM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Import(73000.0)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>M.T.Sargodha</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Pakistan National Ship.Corpt.</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>9/22/2025 10:00:00 PM</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Import(73000.0)</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2025-09-20 06:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Fertilizer / Urea</t>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Shipping Agent</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Arrival Strip</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Import(Tons)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Export(Tons)</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
+          <t>General Cargo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Belita.</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bulk Shipping Agencies Pvt Ltd</t>
+          <t>Shipping Agent</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>9/18/2025 10:30:00 PM</t>
+          <t>Arrival Strip</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Import(40250.0)</t>
+          <t>Import(Tons)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Export(Tons)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>Last Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Xing Ning He</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Seahawks (Pvt) Limited</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>9/19/2025 3:00:00 AM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Import(34820.0)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>General Cargo</t>
+          <t>Ogba</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Ocean Services (Pvt) Ltd</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>9/19/2025 3:45:00 AM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Export(60500.0)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Maritime Amity</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Shipping Agent</t>
+          <t>Alpine Marine Services (Pvt) Ltd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Arrival Strip</t>
+          <t>9/20/2025 4:00:00 PM</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Import(Tons)</t>
+          <t>Import(3800.0)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Export(Tons)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Last Updated</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Xing Ning He</t>
+          <t>Zao Galaxy.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Seahawks (Pvt) Limited</t>
+          <t>Gac Pakistan (Pvt) Limited.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>9/19/2025 3:00:00 AM</t>
+          <t>9/22/2025 8:00:00 AM</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Import(34820.0)</t>
+          <t>Import(2505.0)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1410,103 +1467,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Ogba</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Ocean Services (Pvt) Ltd</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>9/19/2025 3:45:00 AM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Export(60500.0)</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>2025-09-20 06:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Maritime Amity</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Alpine Marine Services (Pvt) Ltd</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>9/20/2025 4:00:00 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Import(3800.0)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2025-09-20 06:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Zao Galaxy.</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Gac Pakistan (Pvt) Limited.</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>9/21/2025 6:00:00 PM</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Import(2505.0)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2025-09-20 06:00:00</t>
+          <t>2025-09-20 20:15:17</t>
         </is>
       </c>
     </row>
@@ -1521,13 +1482,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Updated on Saturday, 20 September 2025;</t>
+          <t>Updated on Sunday, 21 September 2025;</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1563,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:02</t>
+          <t>2025-09-20 20:15:19</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1600,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:02</t>
+          <t>2025-09-20 20:15:19</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1637,81 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:02</t>
+          <t>2025-09-20 20:15:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kota Manzanillo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Container Ship</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pacific Delta Shipping (Pvt) Ltd</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not Allocated</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>9/20/2025 1:48:00 PM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(Planning is already done)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Maritime Amity</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tanker</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Alpine Marine Services (Pvt) Ltd</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Op-2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9/20/2025 5:12:00 PM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(Planning is already done)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2025-09-20 20:15:19</t>
         </is>
       </c>
     </row>
@@ -1691,13 +1726,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Updated on Saturday, 20 September 2025;</t>
+          <t>Updated on Sunday, 21 September 2025;</t>
         </is>
       </c>
     </row>
@@ -1740,44 +1775,6 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Last Updated</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>NAPHTHA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pis Jawa</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Alpine Marine Services (Pvt) Ltd</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>9/19/2025 3:40:00 PM</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KPT-16678</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>183</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2025-09-20 06:00:04</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1795,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Updated on Saturday, 20 September 2025;</t>
+          <t>Updated on Sunday, 21 September 2025;</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1866,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1898,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1930,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1962,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1994,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2026,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2058,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2090,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2122,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2154,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025-09-20 06:00:09</t>
+          <t>2025-09-20 20:15:25</t>
         </is>
       </c>
     </row>

</xml_diff>